<commit_message>
Login, UM, PM Flow Created
</commit_message>
<xml_diff>
--- a/src/test/resources/login_data.xlsx
+++ b/src/test/resources/login_data.xlsx
@@ -54,10 +54,10 @@
     <t>WrongUser</t>
   </si>
   <si>
-    <t>B1350</t>
-  </si>
-  <si>
     <t>Bcil@12345678</t>
+  </si>
+  <si>
+    <t>Test001</t>
   </si>
 </sst>
 </file>
@@ -939,10 +939,10 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>5</v>
@@ -953,7 +953,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>7</v>
@@ -970,7 +970,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>8</v>

</xml_diff>